<commit_message>
feat(pkm-smt3): execute dashboard material remediation
</commit_message>
<xml_diff>
--- a/outputs/2026-10-03-dummy-datasets/dummy-data-agenda-kegiatan-internal.xlsx
+++ b/outputs/2026-10-03-dummy-datasets/dummy-data-agenda-kegiatan-internal.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" r:id="R8a070d430d1a402d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panduan" sheetId="2" r:id="Ra61092ffea834b0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" r:id="R96efe86223b94f9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panduan" sheetId="2" r:id="Rcc9fc9c3b0c640ab"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -53,7 +53,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -73,6 +73,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -215,7 +220,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="45">
+  <x:cellXfs count="48">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -328,8 +333,13 @@
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -606,7 +616,7 @@
         <x:v>AGD-0001</x:v>
       </x:c>
       <x:c r="B2" s="21" t="n">
-        <x:v>46227</x:v>
+        <x:v>46296</x:v>
       </x:c>
       <x:c r="C2" s="15" t="str">
         <x:v>Rapat Koordinasi</x:v>
@@ -615,10 +625,10 @@
         <x:v>Unit D</x:v>
       </x:c>
       <x:c r="E2" s="15" t="str">
-        <x:v>Sosialisasi</x:v>
+        <x:v>Rapat Internal</x:v>
       </x:c>
       <x:c r="F2" s="15" t="str">
-        <x:v>Belum Dimulai</x:v>
+        <x:v>Selesai</x:v>
       </x:c>
       <x:c r="G2" s="15" t="str">
         <x:v>Ruang Rapat 1</x:v>
@@ -641,16 +651,16 @@
         <x:v>AGD-0002</x:v>
       </x:c>
       <x:c r="B3" s="22" t="n">
-        <x:v>46230</x:v>
+        <x:v>46297</x:v>
       </x:c>
       <x:c r="C3" s="18" t="str">
-        <x:v>Evaluasi Bulanan</x:v>
+        <x:v>Sosialisasi Layanan</x:v>
       </x:c>
       <x:c r="D3" s="18" t="str">
         <x:v>Unit A</x:v>
       </x:c>
       <x:c r="E3" s="18" t="str">
-        <x:v>Evaluasi</x:v>
+        <x:v>Sosialisasi</x:v>
       </x:c>
       <x:c r="F3" s="18" t="str">
         <x:v>Selesai</x:v>
@@ -665,7 +675,7 @@
         <x:v>PIC-02</x:v>
       </x:c>
       <x:c r="J3" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K3" s="18" t="str">
         <x:v>Konfirmasi perlengkapan</x:v>
@@ -676,19 +686,19 @@
         <x:v>AGD-0003</x:v>
       </x:c>
       <x:c r="B4" s="22" t="n">
-        <x:v>46233</x:v>
+        <x:v>46298</x:v>
       </x:c>
       <x:c r="C4" s="18" t="str">
-        <x:v>Kegiatan Administrasi</x:v>
+        <x:v>Evaluasi Bulanan</x:v>
       </x:c>
       <x:c r="D4" s="18" t="str">
         <x:v>Unit B</x:v>
       </x:c>
       <x:c r="E4" s="18" t="str">
-        <x:v>Pelatihan</x:v>
+        <x:v>Evaluasi</x:v>
       </x:c>
       <x:c r="F4" s="18" t="str">
-        <x:v>Siap</x:v>
+        <x:v>Selesai</x:v>
       </x:c>
       <x:c r="G4" s="18" t="str">
         <x:v>Ruang Pelayanan</x:v>
@@ -700,7 +710,7 @@
         <x:v>PIC-03</x:v>
       </x:c>
       <x:c r="J4" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K4" s="18" t="str">
         <x:v>Menunggu jadwal final</x:v>
@@ -711,19 +721,19 @@
         <x:v>AGD-0004</x:v>
       </x:c>
       <x:c r="B5" s="22" t="n">
-        <x:v>46236</x:v>
+        <x:v>46296</x:v>
       </x:c>
       <x:c r="C5" s="18" t="str">
-        <x:v>Sosialisasi Layanan</x:v>
+        <x:v>Pelatihan Internal</x:v>
       </x:c>
       <x:c r="D5" s="18" t="str">
         <x:v>Unit C</x:v>
       </x:c>
       <x:c r="E5" s="18" t="str">
-        <x:v>Administrasi</x:v>
+        <x:v>Pelatihan</x:v>
       </x:c>
       <x:c r="F5" s="18" t="str">
-        <x:v>Berjalan</x:v>
+        <x:v>Selesai</x:v>
       </x:c>
       <x:c r="G5" s="18" t="str">
         <x:v>Ruang Rapat 2</x:v>
@@ -746,19 +756,19 @@
         <x:v>AGD-0005</x:v>
       </x:c>
       <x:c r="B6" s="22" t="n">
-        <x:v>46239</x:v>
+        <x:v>46297</x:v>
       </x:c>
       <x:c r="C6" s="18" t="str">
-        <x:v>Pelatihan Internal</x:v>
+        <x:v>Kegiatan Administrasi</x:v>
       </x:c>
       <x:c r="D6" s="18" t="str">
         <x:v>Unit D</x:v>
       </x:c>
       <x:c r="E6" s="18" t="str">
-        <x:v>Rapat Internal</x:v>
+        <x:v>Administrasi</x:v>
       </x:c>
       <x:c r="F6" s="18" t="str">
-        <x:v>Belum Dimulai</x:v>
+        <x:v>Selesai</x:v>
       </x:c>
       <x:c r="G6" s="18" t="str">
         <x:v>Ruang Rapat 1</x:v>
@@ -770,7 +780,7 @@
         <x:v>PIC-05</x:v>
       </x:c>
       <x:c r="J6" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K6" s="18" t="str">
         <x:v>Tidak ada catatan khusus</x:v>
@@ -781,7 +791,7 @@
         <x:v>AGD-0006</x:v>
       </x:c>
       <x:c r="B7" s="22" t="n">
-        <x:v>46242</x:v>
+        <x:v>46298</x:v>
       </x:c>
       <x:c r="C7" s="18" t="str">
         <x:v>Rapat Koordinasi</x:v>
@@ -790,7 +800,7 @@
         <x:v>Unit A</x:v>
       </x:c>
       <x:c r="E7" s="18" t="str">
-        <x:v>Sosialisasi</x:v>
+        <x:v>Rapat Internal</x:v>
       </x:c>
       <x:c r="F7" s="18" t="str">
         <x:v>Selesai</x:v>
@@ -805,7 +815,7 @@
         <x:v>PIC-06</x:v>
       </x:c>
       <x:c r="J7" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K7" s="18" t="str">
         <x:v>Konfirmasi perlengkapan</x:v>
@@ -816,19 +826,19 @@
         <x:v>AGD-0007</x:v>
       </x:c>
       <x:c r="B8" s="22" t="n">
-        <x:v>46245</x:v>
+        <x:v>46296</x:v>
       </x:c>
       <x:c r="C8" s="18" t="str">
-        <x:v>Evaluasi Bulanan</x:v>
+        <x:v>Sosialisasi Layanan</x:v>
       </x:c>
       <x:c r="D8" s="18" t="str">
         <x:v>Unit B</x:v>
       </x:c>
       <x:c r="E8" s="18" t="str">
-        <x:v>Evaluasi</x:v>
+        <x:v>Sosialisasi</x:v>
       </x:c>
       <x:c r="F8" s="18" t="str">
-        <x:v>Siap</x:v>
+        <x:v>Selesai</x:v>
       </x:c>
       <x:c r="G8" s="18" t="str">
         <x:v>Ruang Pelayanan</x:v>
@@ -851,19 +861,19 @@
         <x:v>AGD-0008</x:v>
       </x:c>
       <x:c r="B9" s="22" t="n">
-        <x:v>46248</x:v>
+        <x:v>46297</x:v>
       </x:c>
       <x:c r="C9" s="18" t="str">
-        <x:v>Kegiatan Administrasi</x:v>
+        <x:v>Evaluasi Bulanan</x:v>
       </x:c>
       <x:c r="D9" s="18" t="str">
         <x:v>Unit C</x:v>
       </x:c>
       <x:c r="E9" s="18" t="str">
-        <x:v>Pelatihan</x:v>
+        <x:v>Evaluasi</x:v>
       </x:c>
       <x:c r="F9" s="18" t="str">
-        <x:v>Berjalan</x:v>
+        <x:v>Selesai</x:v>
       </x:c>
       <x:c r="G9" s="18" t="str">
         <x:v>Ruang Rapat 2</x:v>
@@ -875,7 +885,7 @@
         <x:v>PIC-08</x:v>
       </x:c>
       <x:c r="J9" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K9" s="18" t="str">
         <x:v>Data latihan</x:v>
@@ -886,19 +896,19 @@
         <x:v>AGD-0009</x:v>
       </x:c>
       <x:c r="B10" s="22" t="n">
-        <x:v>46251</x:v>
+        <x:v>46298</x:v>
       </x:c>
       <x:c r="C10" s="18" t="str">
-        <x:v>Sosialisasi Layanan</x:v>
+        <x:v>Pelatihan Internal</x:v>
       </x:c>
       <x:c r="D10" s="18" t="str">
         <x:v>Unit D</x:v>
       </x:c>
       <x:c r="E10" s="18" t="str">
-        <x:v>Administrasi</x:v>
+        <x:v>Pelatihan</x:v>
       </x:c>
       <x:c r="F10" s="18" t="str">
-        <x:v>Belum Dimulai</x:v>
+        <x:v>Selesai</x:v>
       </x:c>
       <x:c r="G10" s="18" t="str">
         <x:v>Ruang Rapat 1</x:v>
@@ -910,7 +920,7 @@
         <x:v>PIC-09</x:v>
       </x:c>
       <x:c r="J10" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K10" s="18" t="str">
         <x:v>Tidak ada catatan khusus</x:v>
@@ -921,16 +931,16 @@
         <x:v>AGD-0010</x:v>
       </x:c>
       <x:c r="B11" s="22" t="n">
-        <x:v>46254</x:v>
+        <x:v>46296</x:v>
       </x:c>
       <x:c r="C11" s="18" t="str">
-        <x:v>Pelatihan Internal</x:v>
+        <x:v>Kegiatan Administrasi</x:v>
       </x:c>
       <x:c r="D11" s="18" t="str">
         <x:v>Unit A</x:v>
       </x:c>
       <x:c r="E11" s="18" t="str">
-        <x:v>Rapat Internal</x:v>
+        <x:v>Administrasi</x:v>
       </x:c>
       <x:c r="F11" s="18" t="str">
         <x:v>Selesai</x:v>
@@ -956,7 +966,7 @@
         <x:v>AGD-0011</x:v>
       </x:c>
       <x:c r="B12" s="22" t="n">
-        <x:v>46257</x:v>
+        <x:v>46297</x:v>
       </x:c>
       <x:c r="C12" s="18" t="str">
         <x:v>Rapat Koordinasi</x:v>
@@ -965,10 +975,10 @@
         <x:v>Unit B</x:v>
       </x:c>
       <x:c r="E12" s="18" t="str">
-        <x:v>Sosialisasi</x:v>
+        <x:v>Rapat Internal</x:v>
       </x:c>
       <x:c r="F12" s="18" t="str">
-        <x:v>Siap</x:v>
+        <x:v>Selesai</x:v>
       </x:c>
       <x:c r="G12" s="18" t="str">
         <x:v>Ruang Pelayanan</x:v>
@@ -980,7 +990,7 @@
         <x:v>PIC-11</x:v>
       </x:c>
       <x:c r="J12" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K12" s="18" t="str">
         <x:v>Menunggu jadwal final</x:v>
@@ -991,19 +1001,19 @@
         <x:v>AGD-0012</x:v>
       </x:c>
       <x:c r="B13" s="22" t="n">
-        <x:v>46260</x:v>
+        <x:v>46298</x:v>
       </x:c>
       <x:c r="C13" s="18" t="str">
-        <x:v>Evaluasi Bulanan</x:v>
+        <x:v>Sosialisasi Layanan</x:v>
       </x:c>
       <x:c r="D13" s="18" t="str">
         <x:v>Unit C</x:v>
       </x:c>
       <x:c r="E13" s="18" t="str">
-        <x:v>Evaluasi</x:v>
+        <x:v>Sosialisasi</x:v>
       </x:c>
       <x:c r="F13" s="18" t="str">
-        <x:v>Berjalan</x:v>
+        <x:v>Selesai</x:v>
       </x:c>
       <x:c r="G13" s="18" t="str">
         <x:v>Ruang Rapat 2</x:v>
@@ -1015,7 +1025,7 @@
         <x:v>PIC-12</x:v>
       </x:c>
       <x:c r="J13" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K13" s="18" t="str">
         <x:v>Data latihan</x:v>
@@ -1026,19 +1036,19 @@
         <x:v>AGD-0013</x:v>
       </x:c>
       <x:c r="B14" s="22" t="n">
-        <x:v>46263</x:v>
+        <x:v>46296</x:v>
       </x:c>
       <x:c r="C14" s="18" t="str">
-        <x:v>Kegiatan Administrasi</x:v>
+        <x:v>Evaluasi Bulanan</x:v>
       </x:c>
       <x:c r="D14" s="18" t="str">
         <x:v>Unit D</x:v>
       </x:c>
       <x:c r="E14" s="18" t="str">
-        <x:v>Pelatihan</x:v>
+        <x:v>Evaluasi</x:v>
       </x:c>
       <x:c r="F14" s="18" t="str">
-        <x:v>Belum Dimulai</x:v>
+        <x:v>Selesai</x:v>
       </x:c>
       <x:c r="G14" s="18" t="str">
         <x:v>Ruang Rapat 1</x:v>
@@ -1061,16 +1071,16 @@
         <x:v>AGD-0014</x:v>
       </x:c>
       <x:c r="B15" s="22" t="n">
-        <x:v>46266</x:v>
+        <x:v>46297</x:v>
       </x:c>
       <x:c r="C15" s="18" t="str">
-        <x:v>Sosialisasi Layanan</x:v>
+        <x:v>Pelatihan Internal</x:v>
       </x:c>
       <x:c r="D15" s="18" t="str">
         <x:v>Unit A</x:v>
       </x:c>
       <x:c r="E15" s="18" t="str">
-        <x:v>Administrasi</x:v>
+        <x:v>Pelatihan</x:v>
       </x:c>
       <x:c r="F15" s="18" t="str">
         <x:v>Selesai</x:v>
@@ -1085,7 +1095,7 @@
         <x:v>PIC-02</x:v>
       </x:c>
       <x:c r="J15" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K15" s="18" t="str">
         <x:v>Konfirmasi perlengkapan</x:v>
@@ -1096,19 +1106,19 @@
         <x:v>AGD-0015</x:v>
       </x:c>
       <x:c r="B16" s="22" t="n">
-        <x:v>46269</x:v>
+        <x:v>46298</x:v>
       </x:c>
       <x:c r="C16" s="18" t="str">
-        <x:v>Pelatihan Internal</x:v>
+        <x:v>Kegiatan Administrasi</x:v>
       </x:c>
       <x:c r="D16" s="18" t="str">
         <x:v>Unit B</x:v>
       </x:c>
       <x:c r="E16" s="18" t="str">
-        <x:v>Rapat Internal</x:v>
+        <x:v>Administrasi</x:v>
       </x:c>
       <x:c r="F16" s="18" t="str">
-        <x:v>Siap</x:v>
+        <x:v>Selesai</x:v>
       </x:c>
       <x:c r="G16" s="18" t="str">
         <x:v>Ruang Pelayanan</x:v>
@@ -1120,7 +1130,7 @@
         <x:v>PIC-03</x:v>
       </x:c>
       <x:c r="J16" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K16" s="18" t="str">
         <x:v>Menunggu jadwal final</x:v>
@@ -1131,7 +1141,7 @@
         <x:v>AGD-0016</x:v>
       </x:c>
       <x:c r="B17" s="22" t="n">
-        <x:v>46272</x:v>
+        <x:v>46296</x:v>
       </x:c>
       <x:c r="C17" s="18" t="str">
         <x:v>Rapat Koordinasi</x:v>
@@ -1140,10 +1150,10 @@
         <x:v>Unit C</x:v>
       </x:c>
       <x:c r="E17" s="18" t="str">
-        <x:v>Sosialisasi</x:v>
+        <x:v>Rapat Internal</x:v>
       </x:c>
       <x:c r="F17" s="18" t="str">
-        <x:v>Berjalan</x:v>
+        <x:v>Selesai</x:v>
       </x:c>
       <x:c r="G17" s="18" t="str">
         <x:v>Ruang Rapat 2</x:v>
@@ -1166,19 +1176,19 @@
         <x:v>AGD-0017</x:v>
       </x:c>
       <x:c r="B18" s="22" t="n">
-        <x:v>46275</x:v>
+        <x:v>46297</x:v>
       </x:c>
       <x:c r="C18" s="18" t="str">
-        <x:v>Evaluasi Bulanan</x:v>
+        <x:v>Sosialisasi Layanan</x:v>
       </x:c>
       <x:c r="D18" s="18" t="str">
         <x:v>Unit D</x:v>
       </x:c>
       <x:c r="E18" s="18" t="str">
-        <x:v>Evaluasi</x:v>
+        <x:v>Sosialisasi</x:v>
       </x:c>
       <x:c r="F18" s="18" t="str">
-        <x:v>Belum Dimulai</x:v>
+        <x:v>Selesai</x:v>
       </x:c>
       <x:c r="G18" s="18" t="str">
         <x:v>Ruang Rapat 1</x:v>
@@ -1190,7 +1200,7 @@
         <x:v>PIC-05</x:v>
       </x:c>
       <x:c r="J18" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K18" s="18" t="str">
         <x:v>Tidak ada catatan khusus</x:v>
@@ -1201,16 +1211,16 @@
         <x:v>AGD-0018</x:v>
       </x:c>
       <x:c r="B19" s="22" t="n">
-        <x:v>46278</x:v>
+        <x:v>46298</x:v>
       </x:c>
       <x:c r="C19" s="18" t="str">
-        <x:v>Kegiatan Administrasi</x:v>
+        <x:v>Evaluasi Bulanan</x:v>
       </x:c>
       <x:c r="D19" s="18" t="str">
         <x:v>Unit A</x:v>
       </x:c>
       <x:c r="E19" s="18" t="str">
-        <x:v>Pelatihan</x:v>
+        <x:v>Evaluasi</x:v>
       </x:c>
       <x:c r="F19" s="18" t="str">
         <x:v>Selesai</x:v>
@@ -1225,7 +1235,7 @@
         <x:v>PIC-06</x:v>
       </x:c>
       <x:c r="J19" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K19" s="18" t="str">
         <x:v>Konfirmasi perlengkapan</x:v>
@@ -1236,19 +1246,19 @@
         <x:v>AGD-0019</x:v>
       </x:c>
       <x:c r="B20" s="22" t="n">
-        <x:v>46281</x:v>
+        <x:v>46296</x:v>
       </x:c>
       <x:c r="C20" s="18" t="str">
-        <x:v>Sosialisasi Layanan</x:v>
+        <x:v>Pelatihan Internal</x:v>
       </x:c>
       <x:c r="D20" s="18" t="str">
         <x:v>Unit B</x:v>
       </x:c>
       <x:c r="E20" s="18" t="str">
-        <x:v>Administrasi</x:v>
+        <x:v>Pelatihan</x:v>
       </x:c>
       <x:c r="F20" s="18" t="str">
-        <x:v>Siap</x:v>
+        <x:v>Selesai</x:v>
       </x:c>
       <x:c r="G20" s="18" t="str">
         <x:v>Ruang Pelayanan</x:v>
@@ -1271,19 +1281,19 @@
         <x:v>AGD-0020</x:v>
       </x:c>
       <x:c r="B21" s="22" t="n">
-        <x:v>46284</x:v>
+        <x:v>46297</x:v>
       </x:c>
       <x:c r="C21" s="18" t="str">
-        <x:v>Pelatihan Internal</x:v>
+        <x:v>Kegiatan Administrasi</x:v>
       </x:c>
       <x:c r="D21" s="18" t="str">
         <x:v>Unit C</x:v>
       </x:c>
       <x:c r="E21" s="18" t="str">
-        <x:v>Rapat Internal</x:v>
+        <x:v>Administrasi</x:v>
       </x:c>
       <x:c r="F21" s="18" t="str">
-        <x:v>Berjalan</x:v>
+        <x:v>Selesai</x:v>
       </x:c>
       <x:c r="G21" s="18" t="str">
         <x:v>Ruang Rapat 2</x:v>
@@ -1295,7 +1305,7 @@
         <x:v>PIC-08</x:v>
       </x:c>
       <x:c r="J21" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K21" s="18" t="str">
         <x:v>Data latihan</x:v>
@@ -1306,7 +1316,7 @@
         <x:v>AGD-0021</x:v>
       </x:c>
       <x:c r="B22" s="22" t="n">
-        <x:v>46287</x:v>
+        <x:v>46298</x:v>
       </x:c>
       <x:c r="C22" s="18" t="str">
         <x:v>Rapat Koordinasi</x:v>
@@ -1315,10 +1325,10 @@
         <x:v>Unit D</x:v>
       </x:c>
       <x:c r="E22" s="18" t="str">
-        <x:v>Sosialisasi</x:v>
+        <x:v>Rapat Internal</x:v>
       </x:c>
       <x:c r="F22" s="18" t="str">
-        <x:v>Belum Dimulai</x:v>
+        <x:v>Selesai</x:v>
       </x:c>
       <x:c r="G22" s="18" t="str">
         <x:v>Ruang Rapat 1</x:v>
@@ -1330,7 +1340,7 @@
         <x:v>PIC-09</x:v>
       </x:c>
       <x:c r="J22" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K22" s="18" t="str">
         <x:v>Tidak ada catatan khusus</x:v>
@@ -1341,16 +1351,16 @@
         <x:v>AGD-0022</x:v>
       </x:c>
       <x:c r="B23" s="22" t="n">
-        <x:v>46290</x:v>
+        <x:v>46296</x:v>
       </x:c>
       <x:c r="C23" s="18" t="str">
-        <x:v>Evaluasi Bulanan</x:v>
+        <x:v>Sosialisasi Layanan</x:v>
       </x:c>
       <x:c r="D23" s="18" t="str">
         <x:v>Unit A</x:v>
       </x:c>
       <x:c r="E23" s="18" t="str">
-        <x:v>Evaluasi</x:v>
+        <x:v>Sosialisasi</x:v>
       </x:c>
       <x:c r="F23" s="18" t="str">
         <x:v>Selesai</x:v>
@@ -1376,19 +1386,19 @@
         <x:v>AGD-0023</x:v>
       </x:c>
       <x:c r="B24" s="22" t="n">
-        <x:v>46293</x:v>
+        <x:v>46297</x:v>
       </x:c>
       <x:c r="C24" s="18" t="str">
-        <x:v>Kegiatan Administrasi</x:v>
+        <x:v>Evaluasi Bulanan</x:v>
       </x:c>
       <x:c r="D24" s="18" t="str">
         <x:v>Unit B</x:v>
       </x:c>
       <x:c r="E24" s="18" t="str">
-        <x:v>Pelatihan</x:v>
+        <x:v>Evaluasi</x:v>
       </x:c>
       <x:c r="F24" s="18" t="str">
-        <x:v>Siap</x:v>
+        <x:v>Selesai</x:v>
       </x:c>
       <x:c r="G24" s="18" t="str">
         <x:v>Ruang Pelayanan</x:v>
@@ -1400,7 +1410,7 @@
         <x:v>PIC-11</x:v>
       </x:c>
       <x:c r="J24" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K24" s="18" t="str">
         <x:v>Menunggu jadwal final</x:v>
@@ -1411,19 +1421,19 @@
         <x:v>AGD-0024</x:v>
       </x:c>
       <x:c r="B25" s="22" t="n">
-        <x:v>46296</x:v>
+        <x:v>46298</x:v>
       </x:c>
       <x:c r="C25" s="18" t="str">
-        <x:v>Sosialisasi Layanan</x:v>
+        <x:v>Pelatihan Internal</x:v>
       </x:c>
       <x:c r="D25" s="18" t="str">
         <x:v>Unit C</x:v>
       </x:c>
       <x:c r="E25" s="18" t="str">
-        <x:v>Administrasi</x:v>
+        <x:v>Pelatihan</x:v>
       </x:c>
       <x:c r="F25" s="18" t="str">
-        <x:v>Berjalan</x:v>
+        <x:v>Selesai</x:v>
       </x:c>
       <x:c r="G25" s="18" t="str">
         <x:v>Ruang Rapat 2</x:v>
@@ -1435,7 +1445,7 @@
         <x:v>PIC-12</x:v>
       </x:c>
       <x:c r="J25" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K25" s="18" t="str">
         <x:v>Data latihan</x:v>
@@ -1446,19 +1456,19 @@
         <x:v>AGD-0025</x:v>
       </x:c>
       <x:c r="B26" s="22" t="n">
-        <x:v>46299</x:v>
+        <x:v>46296</x:v>
       </x:c>
       <x:c r="C26" s="18" t="str">
-        <x:v>Pelatihan Internal</x:v>
+        <x:v>Kegiatan Administrasi</x:v>
       </x:c>
       <x:c r="D26" s="18" t="str">
         <x:v>Unit D</x:v>
       </x:c>
       <x:c r="E26" s="18" t="str">
-        <x:v>Rapat Internal</x:v>
+        <x:v>Administrasi</x:v>
       </x:c>
       <x:c r="F26" s="18" t="str">
-        <x:v>Belum Dimulai</x:v>
+        <x:v>Selesai</x:v>
       </x:c>
       <x:c r="G26" s="18" t="str">
         <x:v>Ruang Rapat 1</x:v>
@@ -1481,7 +1491,7 @@
         <x:v>AGD-0026</x:v>
       </x:c>
       <x:c r="B27" s="22" t="n">
-        <x:v>46302</x:v>
+        <x:v>46303</x:v>
       </x:c>
       <x:c r="C27" s="18" t="str">
         <x:v>Rapat Koordinasi</x:v>
@@ -1490,10 +1500,10 @@
         <x:v>Unit A</x:v>
       </x:c>
       <x:c r="E27" s="18" t="str">
-        <x:v>Sosialisasi</x:v>
+        <x:v>Rapat Internal</x:v>
       </x:c>
       <x:c r="F27" s="18" t="str">
-        <x:v>Selesai</x:v>
+        <x:v>Berjalan</x:v>
       </x:c>
       <x:c r="G27" s="18" t="str">
         <x:v>Aula Kecamatan</x:v>
@@ -1505,7 +1515,7 @@
         <x:v>PIC-02</x:v>
       </x:c>
       <x:c r="J27" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K27" s="18" t="str">
         <x:v>Konfirmasi perlengkapan</x:v>
@@ -1516,19 +1526,19 @@
         <x:v>AGD-0027</x:v>
       </x:c>
       <x:c r="B28" s="22" t="n">
-        <x:v>46305</x:v>
+        <x:v>46304</x:v>
       </x:c>
       <x:c r="C28" s="18" t="str">
-        <x:v>Evaluasi Bulanan</x:v>
+        <x:v>Sosialisasi Layanan</x:v>
       </x:c>
       <x:c r="D28" s="18" t="str">
         <x:v>Unit B</x:v>
       </x:c>
       <x:c r="E28" s="18" t="str">
-        <x:v>Evaluasi</x:v>
+        <x:v>Sosialisasi</x:v>
       </x:c>
       <x:c r="F28" s="18" t="str">
-        <x:v>Siap</x:v>
+        <x:v>Berjalan</x:v>
       </x:c>
       <x:c r="G28" s="18" t="str">
         <x:v>Ruang Pelayanan</x:v>
@@ -1540,7 +1550,7 @@
         <x:v>PIC-03</x:v>
       </x:c>
       <x:c r="J28" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K28" s="18" t="str">
         <x:v>Menunggu jadwal final</x:v>
@@ -1551,16 +1561,16 @@
         <x:v>AGD-0028</x:v>
       </x:c>
       <x:c r="B29" s="22" t="n">
-        <x:v>46308</x:v>
+        <x:v>46305</x:v>
       </x:c>
       <x:c r="C29" s="18" t="str">
-        <x:v>Kegiatan Administrasi</x:v>
+        <x:v>Evaluasi Bulanan</x:v>
       </x:c>
       <x:c r="D29" s="18" t="str">
         <x:v>Unit C</x:v>
       </x:c>
       <x:c r="E29" s="18" t="str">
-        <x:v>Pelatihan</x:v>
+        <x:v>Evaluasi</x:v>
       </x:c>
       <x:c r="F29" s="18" t="str">
         <x:v>Berjalan</x:v>
@@ -1586,19 +1596,19 @@
         <x:v>AGD-0029</x:v>
       </x:c>
       <x:c r="B30" s="22" t="n">
-        <x:v>46311</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="C30" s="18" t="str">
-        <x:v>Sosialisasi Layanan</x:v>
+        <x:v>Pelatihan Internal</x:v>
       </x:c>
       <x:c r="D30" s="18" t="str">
         <x:v>Unit D</x:v>
       </x:c>
       <x:c r="E30" s="18" t="str">
-        <x:v>Administrasi</x:v>
+        <x:v>Pelatihan</x:v>
       </x:c>
       <x:c r="F30" s="18" t="str">
-        <x:v>Belum Dimulai</x:v>
+        <x:v>Berjalan</x:v>
       </x:c>
       <x:c r="G30" s="18" t="str">
         <x:v>Ruang Rapat 1</x:v>
@@ -1610,7 +1620,7 @@
         <x:v>PIC-05</x:v>
       </x:c>
       <x:c r="J30" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K30" s="18" t="str">
         <x:v>Tidak ada catatan khusus</x:v>
@@ -1621,19 +1631,19 @@
         <x:v>AGD-0030</x:v>
       </x:c>
       <x:c r="B31" s="22" t="n">
-        <x:v>46314</x:v>
+        <x:v>46300</x:v>
       </x:c>
       <x:c r="C31" s="18" t="str">
-        <x:v>Pelatihan Internal</x:v>
+        <x:v>Kegiatan Administrasi</x:v>
       </x:c>
       <x:c r="D31" s="18" t="str">
         <x:v>Unit A</x:v>
       </x:c>
       <x:c r="E31" s="18" t="str">
-        <x:v>Rapat Internal</x:v>
+        <x:v>Administrasi</x:v>
       </x:c>
       <x:c r="F31" s="18" t="str">
-        <x:v>Selesai</x:v>
+        <x:v>Berjalan</x:v>
       </x:c>
       <x:c r="G31" s="18" t="str">
         <x:v>Aula Kecamatan</x:v>
@@ -1645,7 +1655,7 @@
         <x:v>PIC-06</x:v>
       </x:c>
       <x:c r="J31" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K31" s="18" t="str">
         <x:v>Konfirmasi perlengkapan</x:v>
@@ -1656,7 +1666,7 @@
         <x:v>AGD-0031</x:v>
       </x:c>
       <x:c r="B32" s="22" t="n">
-        <x:v>46317</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="C32" s="18" t="str">
         <x:v>Rapat Koordinasi</x:v>
@@ -1665,10 +1675,10 @@
         <x:v>Unit B</x:v>
       </x:c>
       <x:c r="E32" s="18" t="str">
-        <x:v>Sosialisasi</x:v>
+        <x:v>Rapat Internal</x:v>
       </x:c>
       <x:c r="F32" s="18" t="str">
-        <x:v>Siap</x:v>
+        <x:v>Berjalan</x:v>
       </x:c>
       <x:c r="G32" s="18" t="str">
         <x:v>Ruang Pelayanan</x:v>
@@ -1691,16 +1701,16 @@
         <x:v>AGD-0032</x:v>
       </x:c>
       <x:c r="B33" s="22" t="n">
-        <x:v>46320</x:v>
+        <x:v>46302</x:v>
       </x:c>
       <x:c r="C33" s="18" t="str">
-        <x:v>Evaluasi Bulanan</x:v>
+        <x:v>Sosialisasi Layanan</x:v>
       </x:c>
       <x:c r="D33" s="18" t="str">
         <x:v>Unit C</x:v>
       </x:c>
       <x:c r="E33" s="18" t="str">
-        <x:v>Evaluasi</x:v>
+        <x:v>Sosialisasi</x:v>
       </x:c>
       <x:c r="F33" s="18" t="str">
         <x:v>Berjalan</x:v>
@@ -1715,7 +1725,7 @@
         <x:v>PIC-08</x:v>
       </x:c>
       <x:c r="J33" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K33" s="18" t="str">
         <x:v>Data latihan</x:v>
@@ -1726,19 +1736,19 @@
         <x:v>AGD-0033</x:v>
       </x:c>
       <x:c r="B34" s="22" t="n">
-        <x:v>46053</x:v>
+        <x:v>46303</x:v>
       </x:c>
       <x:c r="C34" s="18" t="str">
-        <x:v>Kegiatan Administrasi</x:v>
+        <x:v>Evaluasi Bulanan</x:v>
       </x:c>
       <x:c r="D34" s="18" t="str">
         <x:v>Unit D</x:v>
       </x:c>
       <x:c r="E34" s="18" t="str">
-        <x:v>Pelatihan</x:v>
+        <x:v>Evaluasi</x:v>
       </x:c>
       <x:c r="F34" s="18" t="str">
-        <x:v>Belum Dimulai</x:v>
+        <x:v>Berjalan</x:v>
       </x:c>
       <x:c r="G34" s="18" t="str">
         <x:v>Ruang Rapat 1</x:v>
@@ -1750,7 +1760,7 @@
         <x:v>PIC-09</x:v>
       </x:c>
       <x:c r="J34" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K34" s="18" t="str">
         <x:v>Tidak ada catatan khusus</x:v>
@@ -1761,19 +1771,19 @@
         <x:v>AGD-0034</x:v>
       </x:c>
       <x:c r="B35" s="22" t="n">
-        <x:v>46056</x:v>
+        <x:v>46304</x:v>
       </x:c>
       <x:c r="C35" s="18" t="str">
-        <x:v>Sosialisasi Layanan</x:v>
+        <x:v>Pelatihan Internal</x:v>
       </x:c>
       <x:c r="D35" s="18" t="str">
         <x:v>Unit A</x:v>
       </x:c>
       <x:c r="E35" s="18" t="str">
-        <x:v>Administrasi</x:v>
+        <x:v>Pelatihan</x:v>
       </x:c>
       <x:c r="F35" s="18" t="str">
-        <x:v>Selesai</x:v>
+        <x:v>Berjalan</x:v>
       </x:c>
       <x:c r="G35" s="18" t="str">
         <x:v>Aula Kecamatan</x:v>
@@ -1796,19 +1806,19 @@
         <x:v>AGD-0035</x:v>
       </x:c>
       <x:c r="B36" s="22" t="n">
-        <x:v>46059</x:v>
+        <x:v>46305</x:v>
       </x:c>
       <x:c r="C36" s="18" t="str">
-        <x:v>Pelatihan Internal</x:v>
+        <x:v>Kegiatan Administrasi</x:v>
       </x:c>
       <x:c r="D36" s="18" t="str">
         <x:v>Unit B</x:v>
       </x:c>
       <x:c r="E36" s="18" t="str">
-        <x:v>Rapat Internal</x:v>
+        <x:v>Administrasi</x:v>
       </x:c>
       <x:c r="F36" s="18" t="str">
-        <x:v>Siap</x:v>
+        <x:v>Berjalan</x:v>
       </x:c>
       <x:c r="G36" s="18" t="str">
         <x:v>Ruang Pelayanan</x:v>
@@ -1820,7 +1830,7 @@
         <x:v>PIC-11</x:v>
       </x:c>
       <x:c r="J36" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K36" s="18" t="str">
         <x:v>Menunggu jadwal final</x:v>
@@ -1831,7 +1841,7 @@
         <x:v>AGD-0036</x:v>
       </x:c>
       <x:c r="B37" s="22" t="n">
-        <x:v>46062</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="C37" s="18" t="str">
         <x:v>Rapat Koordinasi</x:v>
@@ -1840,7 +1850,7 @@
         <x:v>Unit C</x:v>
       </x:c>
       <x:c r="E37" s="18" t="str">
-        <x:v>Sosialisasi</x:v>
+        <x:v>Rapat Internal</x:v>
       </x:c>
       <x:c r="F37" s="18" t="str">
         <x:v>Berjalan</x:v>
@@ -1855,7 +1865,7 @@
         <x:v>PIC-12</x:v>
       </x:c>
       <x:c r="J37" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K37" s="18" t="str">
         <x:v>Data latihan</x:v>
@@ -1866,19 +1876,19 @@
         <x:v>AGD-0037</x:v>
       </x:c>
       <x:c r="B38" s="22" t="n">
-        <x:v>46065</x:v>
+        <x:v>46300</x:v>
       </x:c>
       <x:c r="C38" s="18" t="str">
-        <x:v>Evaluasi Bulanan</x:v>
+        <x:v>Sosialisasi Layanan</x:v>
       </x:c>
       <x:c r="D38" s="18" t="str">
         <x:v>Unit D</x:v>
       </x:c>
       <x:c r="E38" s="18" t="str">
-        <x:v>Evaluasi</x:v>
+        <x:v>Sosialisasi</x:v>
       </x:c>
       <x:c r="F38" s="18" t="str">
-        <x:v>Belum Dimulai</x:v>
+        <x:v>Berjalan</x:v>
       </x:c>
       <x:c r="G38" s="18" t="str">
         <x:v>Ruang Rapat 1</x:v>
@@ -1901,19 +1911,19 @@
         <x:v>AGD-0038</x:v>
       </x:c>
       <x:c r="B39" s="22" t="n">
-        <x:v>46068</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="C39" s="18" t="str">
-        <x:v>Kegiatan Administrasi</x:v>
+        <x:v>Evaluasi Bulanan</x:v>
       </x:c>
       <x:c r="D39" s="18" t="str">
         <x:v>Unit A</x:v>
       </x:c>
       <x:c r="E39" s="18" t="str">
-        <x:v>Pelatihan</x:v>
+        <x:v>Evaluasi</x:v>
       </x:c>
       <x:c r="F39" s="18" t="str">
-        <x:v>Selesai</x:v>
+        <x:v>Berjalan</x:v>
       </x:c>
       <x:c r="G39" s="18" t="str">
         <x:v>Aula Kecamatan</x:v>
@@ -1925,7 +1935,7 @@
         <x:v>PIC-02</x:v>
       </x:c>
       <x:c r="J39" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K39" s="18" t="str">
         <x:v>Konfirmasi perlengkapan</x:v>
@@ -1936,19 +1946,19 @@
         <x:v>AGD-0039</x:v>
       </x:c>
       <x:c r="B40" s="22" t="n">
-        <x:v>46071</x:v>
+        <x:v>46302</x:v>
       </x:c>
       <x:c r="C40" s="18" t="str">
-        <x:v>Sosialisasi Layanan</x:v>
+        <x:v>Pelatihan Internal</x:v>
       </x:c>
       <x:c r="D40" s="18" t="str">
         <x:v>Unit B</x:v>
       </x:c>
       <x:c r="E40" s="18" t="str">
-        <x:v>Administrasi</x:v>
+        <x:v>Pelatihan</x:v>
       </x:c>
       <x:c r="F40" s="18" t="str">
-        <x:v>Siap</x:v>
+        <x:v>Berjalan</x:v>
       </x:c>
       <x:c r="G40" s="18" t="str">
         <x:v>Ruang Pelayanan</x:v>
@@ -1960,7 +1970,7 @@
         <x:v>PIC-03</x:v>
       </x:c>
       <x:c r="J40" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K40" s="18" t="str">
         <x:v>Menunggu jadwal final</x:v>
@@ -1971,16 +1981,16 @@
         <x:v>AGD-0040</x:v>
       </x:c>
       <x:c r="B41" s="22" t="n">
-        <x:v>46074</x:v>
+        <x:v>46303</x:v>
       </x:c>
       <x:c r="C41" s="18" t="str">
-        <x:v>Pelatihan Internal</x:v>
+        <x:v>Kegiatan Administrasi</x:v>
       </x:c>
       <x:c r="D41" s="18" t="str">
         <x:v>Unit C</x:v>
       </x:c>
       <x:c r="E41" s="18" t="str">
-        <x:v>Rapat Internal</x:v>
+        <x:v>Administrasi</x:v>
       </x:c>
       <x:c r="F41" s="18" t="str">
         <x:v>Berjalan</x:v>
@@ -2006,7 +2016,7 @@
         <x:v>AGD-0041</x:v>
       </x:c>
       <x:c r="B42" s="22" t="n">
-        <x:v>46077</x:v>
+        <x:v>46304</x:v>
       </x:c>
       <x:c r="C42" s="18" t="str">
         <x:v>Rapat Koordinasi</x:v>
@@ -2015,10 +2025,10 @@
         <x:v>Unit D</x:v>
       </x:c>
       <x:c r="E42" s="18" t="str">
-        <x:v>Sosialisasi</x:v>
+        <x:v>Rapat Internal</x:v>
       </x:c>
       <x:c r="F42" s="18" t="str">
-        <x:v>Belum Dimulai</x:v>
+        <x:v>Berjalan</x:v>
       </x:c>
       <x:c r="G42" s="18" t="str">
         <x:v>Ruang Rapat 1</x:v>
@@ -2030,7 +2040,7 @@
         <x:v>PIC-05</x:v>
       </x:c>
       <x:c r="J42" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K42" s="18" t="str">
         <x:v>Tidak ada catatan khusus</x:v>
@@ -2041,19 +2051,19 @@
         <x:v>AGD-0042</x:v>
       </x:c>
       <x:c r="B43" s="22" t="n">
-        <x:v>46080</x:v>
+        <x:v>46305</x:v>
       </x:c>
       <x:c r="C43" s="18" t="str">
-        <x:v>Evaluasi Bulanan</x:v>
+        <x:v>Sosialisasi Layanan</x:v>
       </x:c>
       <x:c r="D43" s="18" t="str">
         <x:v>Unit A</x:v>
       </x:c>
       <x:c r="E43" s="18" t="str">
-        <x:v>Evaluasi</x:v>
+        <x:v>Sosialisasi</x:v>
       </x:c>
       <x:c r="F43" s="18" t="str">
-        <x:v>Selesai</x:v>
+        <x:v>Berjalan</x:v>
       </x:c>
       <x:c r="G43" s="18" t="str">
         <x:v>Aula Kecamatan</x:v>
@@ -2065,7 +2075,7 @@
         <x:v>PIC-06</x:v>
       </x:c>
       <x:c r="J43" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K43" s="18" t="str">
         <x:v>Konfirmasi perlengkapan</x:v>
@@ -2076,19 +2086,19 @@
         <x:v>AGD-0043</x:v>
       </x:c>
       <x:c r="B44" s="22" t="n">
-        <x:v>46083</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="C44" s="18" t="str">
-        <x:v>Kegiatan Administrasi</x:v>
+        <x:v>Evaluasi Bulanan</x:v>
       </x:c>
       <x:c r="D44" s="18" t="str">
         <x:v>Unit B</x:v>
       </x:c>
       <x:c r="E44" s="18" t="str">
-        <x:v>Pelatihan</x:v>
+        <x:v>Evaluasi</x:v>
       </x:c>
       <x:c r="F44" s="18" t="str">
-        <x:v>Siap</x:v>
+        <x:v>Berjalan</x:v>
       </x:c>
       <x:c r="G44" s="18" t="str">
         <x:v>Ruang Pelayanan</x:v>
@@ -2111,16 +2121,16 @@
         <x:v>AGD-0044</x:v>
       </x:c>
       <x:c r="B45" s="22" t="n">
-        <x:v>46086</x:v>
+        <x:v>46300</x:v>
       </x:c>
       <x:c r="C45" s="18" t="str">
-        <x:v>Sosialisasi Layanan</x:v>
+        <x:v>Pelatihan Internal</x:v>
       </x:c>
       <x:c r="D45" s="18" t="str">
         <x:v>Unit C</x:v>
       </x:c>
       <x:c r="E45" s="18" t="str">
-        <x:v>Administrasi</x:v>
+        <x:v>Pelatihan</x:v>
       </x:c>
       <x:c r="F45" s="18" t="str">
         <x:v>Berjalan</x:v>
@@ -2135,7 +2145,7 @@
         <x:v>PIC-08</x:v>
       </x:c>
       <x:c r="J45" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K45" s="18" t="str">
         <x:v>Data latihan</x:v>
@@ -2146,19 +2156,19 @@
         <x:v>AGD-0045</x:v>
       </x:c>
       <x:c r="B46" s="22" t="n">
-        <x:v>46089</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="C46" s="18" t="str">
-        <x:v>Pelatihan Internal</x:v>
+        <x:v>Kegiatan Administrasi</x:v>
       </x:c>
       <x:c r="D46" s="18" t="str">
         <x:v>Unit D</x:v>
       </x:c>
       <x:c r="E46" s="18" t="str">
-        <x:v>Rapat Internal</x:v>
+        <x:v>Administrasi</x:v>
       </x:c>
       <x:c r="F46" s="18" t="str">
-        <x:v>Belum Dimulai</x:v>
+        <x:v>Berjalan</x:v>
       </x:c>
       <x:c r="G46" s="18" t="str">
         <x:v>Ruang Rapat 1</x:v>
@@ -2170,7 +2180,7 @@
         <x:v>PIC-09</x:v>
       </x:c>
       <x:c r="J46" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K46" s="18" t="str">
         <x:v>Tidak ada catatan khusus</x:v>
@@ -2181,7 +2191,7 @@
         <x:v>AGD-0046</x:v>
       </x:c>
       <x:c r="B47" s="22" t="n">
-        <x:v>46092</x:v>
+        <x:v>46302</x:v>
       </x:c>
       <x:c r="C47" s="18" t="str">
         <x:v>Rapat Koordinasi</x:v>
@@ -2190,10 +2200,10 @@
         <x:v>Unit A</x:v>
       </x:c>
       <x:c r="E47" s="18" t="str">
-        <x:v>Sosialisasi</x:v>
+        <x:v>Rapat Internal</x:v>
       </x:c>
       <x:c r="F47" s="18" t="str">
-        <x:v>Selesai</x:v>
+        <x:v>Berjalan</x:v>
       </x:c>
       <x:c r="G47" s="18" t="str">
         <x:v>Aula Kecamatan</x:v>
@@ -2216,19 +2226,19 @@
         <x:v>AGD-0047</x:v>
       </x:c>
       <x:c r="B48" s="22" t="n">
-        <x:v>46095</x:v>
+        <x:v>46303</x:v>
       </x:c>
       <x:c r="C48" s="18" t="str">
-        <x:v>Evaluasi Bulanan</x:v>
+        <x:v>Sosialisasi Layanan</x:v>
       </x:c>
       <x:c r="D48" s="18" t="str">
         <x:v>Unit B</x:v>
       </x:c>
       <x:c r="E48" s="18" t="str">
-        <x:v>Evaluasi</x:v>
+        <x:v>Sosialisasi</x:v>
       </x:c>
       <x:c r="F48" s="18" t="str">
-        <x:v>Siap</x:v>
+        <x:v>Berjalan</x:v>
       </x:c>
       <x:c r="G48" s="18" t="str">
         <x:v>Ruang Pelayanan</x:v>
@@ -2240,7 +2250,7 @@
         <x:v>PIC-11</x:v>
       </x:c>
       <x:c r="J48" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K48" s="18" t="str">
         <x:v>Menunggu jadwal final</x:v>
@@ -2251,16 +2261,16 @@
         <x:v>AGD-0048</x:v>
       </x:c>
       <x:c r="B49" s="22" t="n">
-        <x:v>46098</x:v>
+        <x:v>46304</x:v>
       </x:c>
       <x:c r="C49" s="18" t="str">
-        <x:v>Kegiatan Administrasi</x:v>
+        <x:v>Evaluasi Bulanan</x:v>
       </x:c>
       <x:c r="D49" s="18" t="str">
         <x:v>Unit C</x:v>
       </x:c>
       <x:c r="E49" s="18" t="str">
-        <x:v>Pelatihan</x:v>
+        <x:v>Evaluasi</x:v>
       </x:c>
       <x:c r="F49" s="18" t="str">
         <x:v>Berjalan</x:v>
@@ -2275,7 +2285,7 @@
         <x:v>PIC-12</x:v>
       </x:c>
       <x:c r="J49" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K49" s="18" t="str">
         <x:v>Data latihan</x:v>
@@ -2286,19 +2296,19 @@
         <x:v>AGD-0049</x:v>
       </x:c>
       <x:c r="B50" s="22" t="n">
-        <x:v>46101</x:v>
+        <x:v>46305</x:v>
       </x:c>
       <x:c r="C50" s="18" t="str">
-        <x:v>Sosialisasi Layanan</x:v>
+        <x:v>Pelatihan Internal</x:v>
       </x:c>
       <x:c r="D50" s="18" t="str">
         <x:v>Unit D</x:v>
       </x:c>
       <x:c r="E50" s="18" t="str">
-        <x:v>Administrasi</x:v>
+        <x:v>Pelatihan</x:v>
       </x:c>
       <x:c r="F50" s="18" t="str">
-        <x:v>Belum Dimulai</x:v>
+        <x:v>Berjalan</x:v>
       </x:c>
       <x:c r="G50" s="18" t="str">
         <x:v>Ruang Rapat 1</x:v>
@@ -2321,19 +2331,19 @@
         <x:v>AGD-0050</x:v>
       </x:c>
       <x:c r="B51" s="22" t="n">
-        <x:v>46104</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="C51" s="18" t="str">
-        <x:v>Pelatihan Internal</x:v>
+        <x:v>Kegiatan Administrasi</x:v>
       </x:c>
       <x:c r="D51" s="18" t="str">
         <x:v>Unit A</x:v>
       </x:c>
       <x:c r="E51" s="18" t="str">
-        <x:v>Rapat Internal</x:v>
+        <x:v>Administrasi</x:v>
       </x:c>
       <x:c r="F51" s="18" t="str">
-        <x:v>Selesai</x:v>
+        <x:v>Berjalan</x:v>
       </x:c>
       <x:c r="G51" s="18" t="str">
         <x:v>Aula Kecamatan</x:v>
@@ -2345,7 +2355,7 @@
         <x:v>PIC-02</x:v>
       </x:c>
       <x:c r="J51" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K51" s="18" t="str">
         <x:v>Konfirmasi perlengkapan</x:v>
@@ -2356,7 +2366,7 @@
         <x:v>AGD-0051</x:v>
       </x:c>
       <x:c r="B52" s="22" t="n">
-        <x:v>46107</x:v>
+        <x:v>46302</x:v>
       </x:c>
       <x:c r="C52" s="18" t="str">
         <x:v>Rapat Koordinasi</x:v>
@@ -2365,7 +2375,7 @@
         <x:v>Unit B</x:v>
       </x:c>
       <x:c r="E52" s="18" t="str">
-        <x:v>Sosialisasi</x:v>
+        <x:v>Rapat Internal</x:v>
       </x:c>
       <x:c r="F52" s="18" t="str">
         <x:v>Siap</x:v>
@@ -2380,7 +2390,7 @@
         <x:v>PIC-03</x:v>
       </x:c>
       <x:c r="J52" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K52" s="18" t="str">
         <x:v>Menunggu jadwal final</x:v>
@@ -2391,19 +2401,19 @@
         <x:v>AGD-0052</x:v>
       </x:c>
       <x:c r="B53" s="22" t="n">
-        <x:v>46110</x:v>
+        <x:v>46303</x:v>
       </x:c>
       <x:c r="C53" s="18" t="str">
-        <x:v>Evaluasi Bulanan</x:v>
+        <x:v>Sosialisasi Layanan</x:v>
       </x:c>
       <x:c r="D53" s="18" t="str">
         <x:v>Unit C</x:v>
       </x:c>
       <x:c r="E53" s="18" t="str">
-        <x:v>Evaluasi</x:v>
+        <x:v>Sosialisasi</x:v>
       </x:c>
       <x:c r="F53" s="18" t="str">
-        <x:v>Berjalan</x:v>
+        <x:v>Siap</x:v>
       </x:c>
       <x:c r="G53" s="18" t="str">
         <x:v>Ruang Rapat 2</x:v>
@@ -2426,19 +2436,19 @@
         <x:v>AGD-0053</x:v>
       </x:c>
       <x:c r="B54" s="22" t="n">
-        <x:v>46113</x:v>
+        <x:v>46304</x:v>
       </x:c>
       <x:c r="C54" s="18" t="str">
-        <x:v>Kegiatan Administrasi</x:v>
+        <x:v>Evaluasi Bulanan</x:v>
       </x:c>
       <x:c r="D54" s="18" t="str">
         <x:v>Unit D</x:v>
       </x:c>
       <x:c r="E54" s="18" t="str">
-        <x:v>Pelatihan</x:v>
+        <x:v>Evaluasi</x:v>
       </x:c>
       <x:c r="F54" s="18" t="str">
-        <x:v>Belum Dimulai</x:v>
+        <x:v>Siap</x:v>
       </x:c>
       <x:c r="G54" s="18" t="str">
         <x:v>Ruang Rapat 1</x:v>
@@ -2450,7 +2460,7 @@
         <x:v>PIC-05</x:v>
       </x:c>
       <x:c r="J54" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K54" s="18" t="str">
         <x:v>Tidak ada catatan khusus</x:v>
@@ -2461,19 +2471,19 @@
         <x:v>AGD-0054</x:v>
       </x:c>
       <x:c r="B55" s="22" t="n">
-        <x:v>46116</x:v>
+        <x:v>46305</x:v>
       </x:c>
       <x:c r="C55" s="18" t="str">
-        <x:v>Sosialisasi Layanan</x:v>
+        <x:v>Pelatihan Internal</x:v>
       </x:c>
       <x:c r="D55" s="18" t="str">
         <x:v>Unit A</x:v>
       </x:c>
       <x:c r="E55" s="18" t="str">
-        <x:v>Administrasi</x:v>
+        <x:v>Pelatihan</x:v>
       </x:c>
       <x:c r="F55" s="18" t="str">
-        <x:v>Selesai</x:v>
+        <x:v>Siap</x:v>
       </x:c>
       <x:c r="G55" s="18" t="str">
         <x:v>Aula Kecamatan</x:v>
@@ -2485,7 +2495,7 @@
         <x:v>PIC-06</x:v>
       </x:c>
       <x:c r="J55" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K55" s="18" t="str">
         <x:v>Konfirmasi perlengkapan</x:v>
@@ -2496,16 +2506,16 @@
         <x:v>AGD-0055</x:v>
       </x:c>
       <x:c r="B56" s="22" t="n">
-        <x:v>46119</x:v>
+        <x:v>46306</x:v>
       </x:c>
       <x:c r="C56" s="18" t="str">
-        <x:v>Pelatihan Internal</x:v>
+        <x:v>Kegiatan Administrasi</x:v>
       </x:c>
       <x:c r="D56" s="18" t="str">
         <x:v>Unit B</x:v>
       </x:c>
       <x:c r="E56" s="18" t="str">
-        <x:v>Rapat Internal</x:v>
+        <x:v>Administrasi</x:v>
       </x:c>
       <x:c r="F56" s="18" t="str">
         <x:v>Siap</x:v>
@@ -2531,7 +2541,7 @@
         <x:v>AGD-0056</x:v>
       </x:c>
       <x:c r="B57" s="22" t="n">
-        <x:v>46122</x:v>
+        <x:v>46307</x:v>
       </x:c>
       <x:c r="C57" s="18" t="str">
         <x:v>Rapat Koordinasi</x:v>
@@ -2540,10 +2550,10 @@
         <x:v>Unit C</x:v>
       </x:c>
       <x:c r="E57" s="18" t="str">
-        <x:v>Sosialisasi</x:v>
+        <x:v>Rapat Internal</x:v>
       </x:c>
       <x:c r="F57" s="18" t="str">
-        <x:v>Berjalan</x:v>
+        <x:v>Siap</x:v>
       </x:c>
       <x:c r="G57" s="18" t="str">
         <x:v>Ruang Rapat 2</x:v>
@@ -2555,7 +2565,7 @@
         <x:v>PIC-08</x:v>
       </x:c>
       <x:c r="J57" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K57" s="18" t="str">
         <x:v>Data latihan</x:v>
@@ -2566,19 +2576,19 @@
         <x:v>AGD-0057</x:v>
       </x:c>
       <x:c r="B58" s="22" t="n">
-        <x:v>46125</x:v>
+        <x:v>46308</x:v>
       </x:c>
       <x:c r="C58" s="18" t="str">
-        <x:v>Evaluasi Bulanan</x:v>
+        <x:v>Sosialisasi Layanan</x:v>
       </x:c>
       <x:c r="D58" s="18" t="str">
         <x:v>Unit D</x:v>
       </x:c>
       <x:c r="E58" s="18" t="str">
-        <x:v>Evaluasi</x:v>
+        <x:v>Sosialisasi</x:v>
       </x:c>
       <x:c r="F58" s="18" t="str">
-        <x:v>Belum Dimulai</x:v>
+        <x:v>Siap</x:v>
       </x:c>
       <x:c r="G58" s="18" t="str">
         <x:v>Ruang Rapat 1</x:v>
@@ -2590,7 +2600,7 @@
         <x:v>PIC-09</x:v>
       </x:c>
       <x:c r="J58" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K58" s="18" t="str">
         <x:v>Tidak ada catatan khusus</x:v>
@@ -2601,19 +2611,19 @@
         <x:v>AGD-0058</x:v>
       </x:c>
       <x:c r="B59" s="22" t="n">
-        <x:v>46128</x:v>
+        <x:v>46309</x:v>
       </x:c>
       <x:c r="C59" s="18" t="str">
-        <x:v>Kegiatan Administrasi</x:v>
+        <x:v>Evaluasi Bulanan</x:v>
       </x:c>
       <x:c r="D59" s="18" t="str">
         <x:v>Unit A</x:v>
       </x:c>
       <x:c r="E59" s="18" t="str">
-        <x:v>Pelatihan</x:v>
+        <x:v>Evaluasi</x:v>
       </x:c>
       <x:c r="F59" s="18" t="str">
-        <x:v>Selesai</x:v>
+        <x:v>Siap</x:v>
       </x:c>
       <x:c r="G59" s="18" t="str">
         <x:v>Aula Kecamatan</x:v>
@@ -2636,16 +2646,16 @@
         <x:v>AGD-0059</x:v>
       </x:c>
       <x:c r="B60" s="22" t="n">
-        <x:v>46131</x:v>
+        <x:v>46310</x:v>
       </x:c>
       <x:c r="C60" s="18" t="str">
-        <x:v>Sosialisasi Layanan</x:v>
+        <x:v>Pelatihan Internal</x:v>
       </x:c>
       <x:c r="D60" s="18" t="str">
         <x:v>Unit B</x:v>
       </x:c>
       <x:c r="E60" s="18" t="str">
-        <x:v>Administrasi</x:v>
+        <x:v>Pelatihan</x:v>
       </x:c>
       <x:c r="F60" s="18" t="str">
         <x:v>Siap</x:v>
@@ -2660,7 +2670,7 @@
         <x:v>PIC-11</x:v>
       </x:c>
       <x:c r="J60" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K60" s="18" t="str">
         <x:v>Menunggu jadwal final</x:v>
@@ -2671,19 +2681,19 @@
         <x:v>AGD-0060</x:v>
       </x:c>
       <x:c r="B61" s="22" t="n">
-        <x:v>46134</x:v>
+        <x:v>46311</x:v>
       </x:c>
       <x:c r="C61" s="18" t="str">
-        <x:v>Pelatihan Internal</x:v>
+        <x:v>Kegiatan Administrasi</x:v>
       </x:c>
       <x:c r="D61" s="18" t="str">
         <x:v>Unit C</x:v>
       </x:c>
       <x:c r="E61" s="18" t="str">
-        <x:v>Rapat Internal</x:v>
+        <x:v>Administrasi</x:v>
       </x:c>
       <x:c r="F61" s="18" t="str">
-        <x:v>Berjalan</x:v>
+        <x:v>Siap</x:v>
       </x:c>
       <x:c r="G61" s="18" t="str">
         <x:v>Ruang Rapat 2</x:v>
@@ -2695,7 +2705,7 @@
         <x:v>PIC-12</x:v>
       </x:c>
       <x:c r="J61" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K61" s="18" t="str">
         <x:v>Data latihan</x:v>
@@ -2706,7 +2716,7 @@
         <x:v>AGD-0061</x:v>
       </x:c>
       <x:c r="B62" s="22" t="n">
-        <x:v>46137</x:v>
+        <x:v>46312</x:v>
       </x:c>
       <x:c r="C62" s="18" t="str">
         <x:v>Rapat Koordinasi</x:v>
@@ -2715,10 +2725,10 @@
         <x:v>Unit D</x:v>
       </x:c>
       <x:c r="E62" s="18" t="str">
-        <x:v>Sosialisasi</x:v>
+        <x:v>Rapat Internal</x:v>
       </x:c>
       <x:c r="F62" s="18" t="str">
-        <x:v>Belum Dimulai</x:v>
+        <x:v>Siap</x:v>
       </x:c>
       <x:c r="G62" s="18" t="str">
         <x:v>Ruang Rapat 1</x:v>
@@ -2741,19 +2751,19 @@
         <x:v>AGD-0062</x:v>
       </x:c>
       <x:c r="B63" s="22" t="n">
-        <x:v>46140</x:v>
+        <x:v>46313</x:v>
       </x:c>
       <x:c r="C63" s="18" t="str">
-        <x:v>Evaluasi Bulanan</x:v>
+        <x:v>Sosialisasi Layanan</x:v>
       </x:c>
       <x:c r="D63" s="18" t="str">
         <x:v>Unit A</x:v>
       </x:c>
       <x:c r="E63" s="18" t="str">
-        <x:v>Evaluasi</x:v>
+        <x:v>Sosialisasi</x:v>
       </x:c>
       <x:c r="F63" s="18" t="str">
-        <x:v>Selesai</x:v>
+        <x:v>Siap</x:v>
       </x:c>
       <x:c r="G63" s="18" t="str">
         <x:v>Aula Kecamatan</x:v>
@@ -2765,7 +2775,7 @@
         <x:v>PIC-02</x:v>
       </x:c>
       <x:c r="J63" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K63" s="18" t="str">
         <x:v>Konfirmasi perlengkapan</x:v>
@@ -2776,16 +2786,16 @@
         <x:v>AGD-0063</x:v>
       </x:c>
       <x:c r="B64" s="22" t="n">
-        <x:v>46143</x:v>
+        <x:v>46314</x:v>
       </x:c>
       <x:c r="C64" s="18" t="str">
-        <x:v>Kegiatan Administrasi</x:v>
+        <x:v>Evaluasi Bulanan</x:v>
       </x:c>
       <x:c r="D64" s="18" t="str">
         <x:v>Unit B</x:v>
       </x:c>
       <x:c r="E64" s="18" t="str">
-        <x:v>Pelatihan</x:v>
+        <x:v>Evaluasi</x:v>
       </x:c>
       <x:c r="F64" s="18" t="str">
         <x:v>Siap</x:v>
@@ -2800,7 +2810,7 @@
         <x:v>PIC-03</x:v>
       </x:c>
       <x:c r="J64" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K64" s="18" t="str">
         <x:v>Menunggu jadwal final</x:v>
@@ -2811,19 +2821,19 @@
         <x:v>AGD-0064</x:v>
       </x:c>
       <x:c r="B65" s="22" t="n">
-        <x:v>46146</x:v>
+        <x:v>46315</x:v>
       </x:c>
       <x:c r="C65" s="18" t="str">
-        <x:v>Sosialisasi Layanan</x:v>
+        <x:v>Pelatihan Internal</x:v>
       </x:c>
       <x:c r="D65" s="18" t="str">
         <x:v>Unit C</x:v>
       </x:c>
       <x:c r="E65" s="18" t="str">
-        <x:v>Administrasi</x:v>
+        <x:v>Pelatihan</x:v>
       </x:c>
       <x:c r="F65" s="18" t="str">
-        <x:v>Berjalan</x:v>
+        <x:v>Siap</x:v>
       </x:c>
       <x:c r="G65" s="18" t="str">
         <x:v>Ruang Rapat 2</x:v>
@@ -2846,19 +2856,19 @@
         <x:v>AGD-0065</x:v>
       </x:c>
       <x:c r="B66" s="22" t="n">
-        <x:v>46149</x:v>
+        <x:v>46300</x:v>
       </x:c>
       <x:c r="C66" s="18" t="str">
-        <x:v>Pelatihan Internal</x:v>
+        <x:v>Kegiatan Administrasi</x:v>
       </x:c>
       <x:c r="D66" s="18" t="str">
         <x:v>Unit D</x:v>
       </x:c>
       <x:c r="E66" s="18" t="str">
-        <x:v>Rapat Internal</x:v>
+        <x:v>Administrasi</x:v>
       </x:c>
       <x:c r="F66" s="18" t="str">
-        <x:v>Belum Dimulai</x:v>
+        <x:v>Siap</x:v>
       </x:c>
       <x:c r="G66" s="18" t="str">
         <x:v>Ruang Rapat 1</x:v>
@@ -2870,7 +2880,7 @@
         <x:v>PIC-05</x:v>
       </x:c>
       <x:c r="J66" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K66" s="18" t="str">
         <x:v>Tidak ada catatan khusus</x:v>
@@ -2881,7 +2891,7 @@
         <x:v>AGD-0066</x:v>
       </x:c>
       <x:c r="B67" s="22" t="n">
-        <x:v>46152</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="C67" s="18" t="str">
         <x:v>Rapat Koordinasi</x:v>
@@ -2890,10 +2900,10 @@
         <x:v>Unit A</x:v>
       </x:c>
       <x:c r="E67" s="18" t="str">
-        <x:v>Sosialisasi</x:v>
+        <x:v>Rapat Internal</x:v>
       </x:c>
       <x:c r="F67" s="18" t="str">
-        <x:v>Selesai</x:v>
+        <x:v>Siap</x:v>
       </x:c>
       <x:c r="G67" s="18" t="str">
         <x:v>Aula Kecamatan</x:v>
@@ -2905,7 +2915,7 @@
         <x:v>PIC-06</x:v>
       </x:c>
       <x:c r="J67" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K67" s="18" t="str">
         <x:v>Konfirmasi perlengkapan</x:v>
@@ -2916,16 +2926,16 @@
         <x:v>AGD-0067</x:v>
       </x:c>
       <x:c r="B68" s="22" t="n">
-        <x:v>46155</x:v>
+        <x:v>46302</x:v>
       </x:c>
       <x:c r="C68" s="18" t="str">
-        <x:v>Evaluasi Bulanan</x:v>
+        <x:v>Sosialisasi Layanan</x:v>
       </x:c>
       <x:c r="D68" s="18" t="str">
         <x:v>Unit B</x:v>
       </x:c>
       <x:c r="E68" s="18" t="str">
-        <x:v>Evaluasi</x:v>
+        <x:v>Sosialisasi</x:v>
       </x:c>
       <x:c r="F68" s="18" t="str">
         <x:v>Siap</x:v>
@@ -2951,19 +2961,19 @@
         <x:v>AGD-0068</x:v>
       </x:c>
       <x:c r="B69" s="22" t="n">
-        <x:v>46158</x:v>
+        <x:v>46303</x:v>
       </x:c>
       <x:c r="C69" s="18" t="str">
-        <x:v>Kegiatan Administrasi</x:v>
+        <x:v>Evaluasi Bulanan</x:v>
       </x:c>
       <x:c r="D69" s="18" t="str">
         <x:v>Unit C</x:v>
       </x:c>
       <x:c r="E69" s="18" t="str">
-        <x:v>Pelatihan</x:v>
+        <x:v>Evaluasi</x:v>
       </x:c>
       <x:c r="F69" s="18" t="str">
-        <x:v>Berjalan</x:v>
+        <x:v>Siap</x:v>
       </x:c>
       <x:c r="G69" s="18" t="str">
         <x:v>Ruang Rapat 2</x:v>
@@ -2975,7 +2985,7 @@
         <x:v>PIC-08</x:v>
       </x:c>
       <x:c r="J69" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K69" s="18" t="str">
         <x:v>Data latihan</x:v>
@@ -2986,19 +2996,19 @@
         <x:v>AGD-0069</x:v>
       </x:c>
       <x:c r="B70" s="22" t="n">
-        <x:v>46161</x:v>
+        <x:v>46304</x:v>
       </x:c>
       <x:c r="C70" s="18" t="str">
-        <x:v>Sosialisasi Layanan</x:v>
+        <x:v>Pelatihan Internal</x:v>
       </x:c>
       <x:c r="D70" s="18" t="str">
         <x:v>Unit D</x:v>
       </x:c>
       <x:c r="E70" s="18" t="str">
-        <x:v>Administrasi</x:v>
+        <x:v>Pelatihan</x:v>
       </x:c>
       <x:c r="F70" s="18" t="str">
-        <x:v>Belum Dimulai</x:v>
+        <x:v>Siap</x:v>
       </x:c>
       <x:c r="G70" s="18" t="str">
         <x:v>Ruang Rapat 1</x:v>
@@ -3010,7 +3020,7 @@
         <x:v>PIC-09</x:v>
       </x:c>
       <x:c r="J70" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K70" s="18" t="str">
         <x:v>Tidak ada catatan khusus</x:v>
@@ -3021,19 +3031,19 @@
         <x:v>AGD-0070</x:v>
       </x:c>
       <x:c r="B71" s="22" t="n">
-        <x:v>46164</x:v>
+        <x:v>46305</x:v>
       </x:c>
       <x:c r="C71" s="18" t="str">
-        <x:v>Pelatihan Internal</x:v>
+        <x:v>Kegiatan Administrasi</x:v>
       </x:c>
       <x:c r="D71" s="18" t="str">
         <x:v>Unit A</x:v>
       </x:c>
       <x:c r="E71" s="18" t="str">
-        <x:v>Rapat Internal</x:v>
+        <x:v>Administrasi</x:v>
       </x:c>
       <x:c r="F71" s="18" t="str">
-        <x:v>Selesai</x:v>
+        <x:v>Siap</x:v>
       </x:c>
       <x:c r="G71" s="18" t="str">
         <x:v>Aula Kecamatan</x:v>
@@ -3056,7 +3066,7 @@
         <x:v>AGD-0071</x:v>
       </x:c>
       <x:c r="B72" s="22" t="n">
-        <x:v>46167</x:v>
+        <x:v>46306</x:v>
       </x:c>
       <x:c r="C72" s="18" t="str">
         <x:v>Rapat Koordinasi</x:v>
@@ -3065,7 +3075,7 @@
         <x:v>Unit B</x:v>
       </x:c>
       <x:c r="E72" s="18" t="str">
-        <x:v>Sosialisasi</x:v>
+        <x:v>Rapat Internal</x:v>
       </x:c>
       <x:c r="F72" s="18" t="str">
         <x:v>Siap</x:v>
@@ -3080,7 +3090,7 @@
         <x:v>PIC-11</x:v>
       </x:c>
       <x:c r="J72" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K72" s="18" t="str">
         <x:v>Menunggu jadwal final</x:v>
@@ -3091,19 +3101,19 @@
         <x:v>AGD-0072</x:v>
       </x:c>
       <x:c r="B73" s="22" t="n">
-        <x:v>46170</x:v>
+        <x:v>46307</x:v>
       </x:c>
       <x:c r="C73" s="18" t="str">
-        <x:v>Evaluasi Bulanan</x:v>
+        <x:v>Sosialisasi Layanan</x:v>
       </x:c>
       <x:c r="D73" s="18" t="str">
         <x:v>Unit C</x:v>
       </x:c>
       <x:c r="E73" s="18" t="str">
-        <x:v>Evaluasi</x:v>
+        <x:v>Sosialisasi</x:v>
       </x:c>
       <x:c r="F73" s="18" t="str">
-        <x:v>Berjalan</x:v>
+        <x:v>Siap</x:v>
       </x:c>
       <x:c r="G73" s="18" t="str">
         <x:v>Ruang Rapat 2</x:v>
@@ -3115,7 +3125,7 @@
         <x:v>PIC-12</x:v>
       </x:c>
       <x:c r="J73" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K73" s="18" t="str">
         <x:v>Data latihan</x:v>
@@ -3126,19 +3136,19 @@
         <x:v>AGD-0073</x:v>
       </x:c>
       <x:c r="B74" s="22" t="n">
-        <x:v>46173</x:v>
+        <x:v>46308</x:v>
       </x:c>
       <x:c r="C74" s="18" t="str">
-        <x:v>Kegiatan Administrasi</x:v>
+        <x:v>Evaluasi Bulanan</x:v>
       </x:c>
       <x:c r="D74" s="18" t="str">
         <x:v>Unit D</x:v>
       </x:c>
       <x:c r="E74" s="18" t="str">
-        <x:v>Pelatihan</x:v>
+        <x:v>Evaluasi</x:v>
       </x:c>
       <x:c r="F74" s="18" t="str">
-        <x:v>Belum Dimulai</x:v>
+        <x:v>Siap</x:v>
       </x:c>
       <x:c r="G74" s="18" t="str">
         <x:v>Ruang Rapat 1</x:v>
@@ -3161,19 +3171,19 @@
         <x:v>AGD-0074</x:v>
       </x:c>
       <x:c r="B75" s="22" t="n">
-        <x:v>46176</x:v>
+        <x:v>46309</x:v>
       </x:c>
       <x:c r="C75" s="18" t="str">
-        <x:v>Sosialisasi Layanan</x:v>
+        <x:v>Pelatihan Internal</x:v>
       </x:c>
       <x:c r="D75" s="18" t="str">
         <x:v>Unit A</x:v>
       </x:c>
       <x:c r="E75" s="18" t="str">
-        <x:v>Administrasi</x:v>
+        <x:v>Pelatihan</x:v>
       </x:c>
       <x:c r="F75" s="18" t="str">
-        <x:v>Selesai</x:v>
+        <x:v>Siap</x:v>
       </x:c>
       <x:c r="G75" s="18" t="str">
         <x:v>Aula Kecamatan</x:v>
@@ -3185,7 +3195,7 @@
         <x:v>PIC-02</x:v>
       </x:c>
       <x:c r="J75" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K75" s="18" t="str">
         <x:v>Konfirmasi perlengkapan</x:v>
@@ -3196,16 +3206,16 @@
         <x:v>AGD-0075</x:v>
       </x:c>
       <x:c r="B76" s="22" t="n">
-        <x:v>46179</x:v>
+        <x:v>46310</x:v>
       </x:c>
       <x:c r="C76" s="18" t="str">
-        <x:v>Pelatihan Internal</x:v>
+        <x:v>Kegiatan Administrasi</x:v>
       </x:c>
       <x:c r="D76" s="18" t="str">
         <x:v>Unit B</x:v>
       </x:c>
       <x:c r="E76" s="18" t="str">
-        <x:v>Rapat Internal</x:v>
+        <x:v>Administrasi</x:v>
       </x:c>
       <x:c r="F76" s="18" t="str">
         <x:v>Siap</x:v>
@@ -3220,7 +3230,7 @@
         <x:v>PIC-03</x:v>
       </x:c>
       <x:c r="J76" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K76" s="18" t="str">
         <x:v>Menunggu jadwal final</x:v>
@@ -3231,7 +3241,7 @@
         <x:v>AGD-0076</x:v>
       </x:c>
       <x:c r="B77" s="22" t="n">
-        <x:v>46182</x:v>
+        <x:v>46321</x:v>
       </x:c>
       <x:c r="C77" s="18" t="str">
         <x:v>Rapat Koordinasi</x:v>
@@ -3240,10 +3250,10 @@
         <x:v>Unit C</x:v>
       </x:c>
       <x:c r="E77" s="18" t="str">
-        <x:v>Sosialisasi</x:v>
+        <x:v>Rapat Internal</x:v>
       </x:c>
       <x:c r="F77" s="18" t="str">
-        <x:v>Berjalan</x:v>
+        <x:v>Belum Dimulai</x:v>
       </x:c>
       <x:c r="G77" s="18" t="str">
         <x:v>Ruang Rapat 2</x:v>
@@ -3266,16 +3276,16 @@
         <x:v>AGD-0077</x:v>
       </x:c>
       <x:c r="B78" s="22" t="n">
-        <x:v>46185</x:v>
+        <x:v>46322</x:v>
       </x:c>
       <x:c r="C78" s="18" t="str">
-        <x:v>Evaluasi Bulanan</x:v>
+        <x:v>Sosialisasi Layanan</x:v>
       </x:c>
       <x:c r="D78" s="18" t="str">
         <x:v>Unit D</x:v>
       </x:c>
       <x:c r="E78" s="18" t="str">
-        <x:v>Evaluasi</x:v>
+        <x:v>Sosialisasi</x:v>
       </x:c>
       <x:c r="F78" s="18" t="str">
         <x:v>Belum Dimulai</x:v>
@@ -3290,7 +3300,7 @@
         <x:v>PIC-05</x:v>
       </x:c>
       <x:c r="J78" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K78" s="18" t="str">
         <x:v>Tidak ada catatan khusus</x:v>
@@ -3301,19 +3311,19 @@
         <x:v>AGD-0078</x:v>
       </x:c>
       <x:c r="B79" s="22" t="n">
-        <x:v>46188</x:v>
+        <x:v>46323</x:v>
       </x:c>
       <x:c r="C79" s="18" t="str">
-        <x:v>Kegiatan Administrasi</x:v>
+        <x:v>Evaluasi Bulanan</x:v>
       </x:c>
       <x:c r="D79" s="18" t="str">
         <x:v>Unit A</x:v>
       </x:c>
       <x:c r="E79" s="18" t="str">
-        <x:v>Pelatihan</x:v>
+        <x:v>Evaluasi</x:v>
       </x:c>
       <x:c r="F79" s="18" t="str">
-        <x:v>Selesai</x:v>
+        <x:v>Belum Dimulai</x:v>
       </x:c>
       <x:c r="G79" s="18" t="str">
         <x:v>Aula Kecamatan</x:v>
@@ -3325,7 +3335,7 @@
         <x:v>PIC-06</x:v>
       </x:c>
       <x:c r="J79" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K79" s="18" t="str">
         <x:v>Konfirmasi perlengkapan</x:v>
@@ -3336,19 +3346,19 @@
         <x:v>AGD-0079</x:v>
       </x:c>
       <x:c r="B80" s="22" t="n">
-        <x:v>46191</x:v>
+        <x:v>46324</x:v>
       </x:c>
       <x:c r="C80" s="18" t="str">
-        <x:v>Sosialisasi Layanan</x:v>
+        <x:v>Pelatihan Internal</x:v>
       </x:c>
       <x:c r="D80" s="18" t="str">
         <x:v>Unit B</x:v>
       </x:c>
       <x:c r="E80" s="18" t="str">
-        <x:v>Administrasi</x:v>
+        <x:v>Pelatihan</x:v>
       </x:c>
       <x:c r="F80" s="18" t="str">
-        <x:v>Siap</x:v>
+        <x:v>Belum Dimulai</x:v>
       </x:c>
       <x:c r="G80" s="18" t="str">
         <x:v>Ruang Pelayanan</x:v>
@@ -3371,19 +3381,19 @@
         <x:v>AGD-0080</x:v>
       </x:c>
       <x:c r="B81" s="22" t="n">
-        <x:v>46194</x:v>
+        <x:v>46325</x:v>
       </x:c>
       <x:c r="C81" s="18" t="str">
-        <x:v>Pelatihan Internal</x:v>
+        <x:v>Kegiatan Administrasi</x:v>
       </x:c>
       <x:c r="D81" s="18" t="str">
         <x:v>Unit C</x:v>
       </x:c>
       <x:c r="E81" s="18" t="str">
-        <x:v>Rapat Internal</x:v>
+        <x:v>Administrasi</x:v>
       </x:c>
       <x:c r="F81" s="18" t="str">
-        <x:v>Berjalan</x:v>
+        <x:v>Belum Dimulai</x:v>
       </x:c>
       <x:c r="G81" s="18" t="str">
         <x:v>Ruang Rapat 2</x:v>
@@ -3395,7 +3405,7 @@
         <x:v>PIC-08</x:v>
       </x:c>
       <x:c r="J81" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K81" s="18" t="str">
         <x:v>Data latihan</x:v>
@@ -3406,7 +3416,7 @@
         <x:v>AGD-0081</x:v>
       </x:c>
       <x:c r="B82" s="22" t="n">
-        <x:v>46197</x:v>
+        <x:v>46306</x:v>
       </x:c>
       <x:c r="C82" s="18" t="str">
         <x:v>Rapat Koordinasi</x:v>
@@ -3415,7 +3425,7 @@
         <x:v>Unit D</x:v>
       </x:c>
       <x:c r="E82" s="18" t="str">
-        <x:v>Sosialisasi</x:v>
+        <x:v>Rapat Internal</x:v>
       </x:c>
       <x:c r="F82" s="18" t="str">
         <x:v>Belum Dimulai</x:v>
@@ -3430,7 +3440,7 @@
         <x:v>PIC-09</x:v>
       </x:c>
       <x:c r="J82" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K82" s="18" t="str">
         <x:v>Tidak ada catatan khusus</x:v>
@@ -3441,19 +3451,19 @@
         <x:v>AGD-0082</x:v>
       </x:c>
       <x:c r="B83" s="22" t="n">
-        <x:v>46200</x:v>
+        <x:v>46307</x:v>
       </x:c>
       <x:c r="C83" s="18" t="str">
-        <x:v>Evaluasi Bulanan</x:v>
+        <x:v>Sosialisasi Layanan</x:v>
       </x:c>
       <x:c r="D83" s="18" t="str">
         <x:v>Unit A</x:v>
       </x:c>
       <x:c r="E83" s="18" t="str">
-        <x:v>Evaluasi</x:v>
+        <x:v>Sosialisasi</x:v>
       </x:c>
       <x:c r="F83" s="18" t="str">
-        <x:v>Selesai</x:v>
+        <x:v>Belum Dimulai</x:v>
       </x:c>
       <x:c r="G83" s="18" t="str">
         <x:v>Aula Kecamatan</x:v>
@@ -3476,19 +3486,19 @@
         <x:v>AGD-0083</x:v>
       </x:c>
       <x:c r="B84" s="22" t="n">
-        <x:v>46203</x:v>
+        <x:v>46308</x:v>
       </x:c>
       <x:c r="C84" s="18" t="str">
-        <x:v>Kegiatan Administrasi</x:v>
+        <x:v>Evaluasi Bulanan</x:v>
       </x:c>
       <x:c r="D84" s="18" t="str">
         <x:v>Unit B</x:v>
       </x:c>
       <x:c r="E84" s="18" t="str">
-        <x:v>Pelatihan</x:v>
+        <x:v>Evaluasi</x:v>
       </x:c>
       <x:c r="F84" s="18" t="str">
-        <x:v>Siap</x:v>
+        <x:v>Belum Dimulai</x:v>
       </x:c>
       <x:c r="G84" s="18" t="str">
         <x:v>Ruang Pelayanan</x:v>
@@ -3500,7 +3510,7 @@
         <x:v>PIC-11</x:v>
       </x:c>
       <x:c r="J84" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K84" s="18" t="str">
         <x:v>Menunggu jadwal final</x:v>
@@ -3511,19 +3521,19 @@
         <x:v>AGD-0084</x:v>
       </x:c>
       <x:c r="B85" s="22" t="n">
-        <x:v>46206</x:v>
+        <x:v>46309</x:v>
       </x:c>
       <x:c r="C85" s="18" t="str">
-        <x:v>Sosialisasi Layanan</x:v>
+        <x:v>Pelatihan Internal</x:v>
       </x:c>
       <x:c r="D85" s="18" t="str">
         <x:v>Unit C</x:v>
       </x:c>
       <x:c r="E85" s="18" t="str">
-        <x:v>Administrasi</x:v>
+        <x:v>Pelatihan</x:v>
       </x:c>
       <x:c r="F85" s="18" t="str">
-        <x:v>Berjalan</x:v>
+        <x:v>Belum Dimulai</x:v>
       </x:c>
       <x:c r="G85" s="18" t="str">
         <x:v>Ruang Rapat 2</x:v>
@@ -3535,7 +3545,7 @@
         <x:v>PIC-12</x:v>
       </x:c>
       <x:c r="J85" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K85" s="18" t="str">
         <x:v>Data latihan</x:v>
@@ -3546,16 +3556,16 @@
         <x:v>AGD-0085</x:v>
       </x:c>
       <x:c r="B86" s="22" t="n">
-        <x:v>46209</x:v>
+        <x:v>46310</x:v>
       </x:c>
       <x:c r="C86" s="18" t="str">
-        <x:v>Pelatihan Internal</x:v>
+        <x:v>Kegiatan Administrasi</x:v>
       </x:c>
       <x:c r="D86" s="18" t="str">
         <x:v>Unit D</x:v>
       </x:c>
       <x:c r="E86" s="18" t="str">
-        <x:v>Rapat Internal</x:v>
+        <x:v>Administrasi</x:v>
       </x:c>
       <x:c r="F86" s="18" t="str">
         <x:v>Belum Dimulai</x:v>
@@ -3581,7 +3591,7 @@
         <x:v>AGD-0086</x:v>
       </x:c>
       <x:c r="B87" s="22" t="n">
-        <x:v>46212</x:v>
+        <x:v>46311</x:v>
       </x:c>
       <x:c r="C87" s="18" t="str">
         <x:v>Rapat Koordinasi</x:v>
@@ -3590,10 +3600,10 @@
         <x:v>Unit A</x:v>
       </x:c>
       <x:c r="E87" s="18" t="str">
-        <x:v>Sosialisasi</x:v>
+        <x:v>Rapat Internal</x:v>
       </x:c>
       <x:c r="F87" s="18" t="str">
-        <x:v>Selesai</x:v>
+        <x:v>Belum Dimulai</x:v>
       </x:c>
       <x:c r="G87" s="18" t="str">
         <x:v>Aula Kecamatan</x:v>
@@ -3605,7 +3615,7 @@
         <x:v>PIC-02</x:v>
       </x:c>
       <x:c r="J87" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K87" s="18" t="str">
         <x:v>Konfirmasi perlengkapan</x:v>
@@ -3616,19 +3626,19 @@
         <x:v>AGD-0087</x:v>
       </x:c>
       <x:c r="B88" s="22" t="n">
-        <x:v>46215</x:v>
+        <x:v>46312</x:v>
       </x:c>
       <x:c r="C88" s="18" t="str">
-        <x:v>Evaluasi Bulanan</x:v>
+        <x:v>Sosialisasi Layanan</x:v>
       </x:c>
       <x:c r="D88" s="18" t="str">
         <x:v>Unit B</x:v>
       </x:c>
       <x:c r="E88" s="18" t="str">
-        <x:v>Evaluasi</x:v>
+        <x:v>Sosialisasi</x:v>
       </x:c>
       <x:c r="F88" s="18" t="str">
-        <x:v>Siap</x:v>
+        <x:v>Belum Dimulai</x:v>
       </x:c>
       <x:c r="G88" s="18" t="str">
         <x:v>Ruang Pelayanan</x:v>
@@ -3640,7 +3650,7 @@
         <x:v>PIC-03</x:v>
       </x:c>
       <x:c r="J88" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K88" s="18" t="str">
         <x:v>Menunggu jadwal final</x:v>
@@ -3651,19 +3661,19 @@
         <x:v>AGD-0088</x:v>
       </x:c>
       <x:c r="B89" s="22" t="n">
-        <x:v>46218</x:v>
+        <x:v>46313</x:v>
       </x:c>
       <x:c r="C89" s="18" t="str">
-        <x:v>Kegiatan Administrasi</x:v>
+        <x:v>Evaluasi Bulanan</x:v>
       </x:c>
       <x:c r="D89" s="18" t="str">
         <x:v>Unit C</x:v>
       </x:c>
       <x:c r="E89" s="18" t="str">
-        <x:v>Pelatihan</x:v>
+        <x:v>Evaluasi</x:v>
       </x:c>
       <x:c r="F89" s="18" t="str">
-        <x:v>Berjalan</x:v>
+        <x:v>Belum Dimulai</x:v>
       </x:c>
       <x:c r="G89" s="18" t="str">
         <x:v>Ruang Rapat 2</x:v>
@@ -3686,16 +3696,16 @@
         <x:v>AGD-0089</x:v>
       </x:c>
       <x:c r="B90" s="22" t="n">
-        <x:v>46221</x:v>
+        <x:v>46314</x:v>
       </x:c>
       <x:c r="C90" s="18" t="str">
-        <x:v>Sosialisasi Layanan</x:v>
+        <x:v>Pelatihan Internal</x:v>
       </x:c>
       <x:c r="D90" s="18" t="str">
         <x:v>Unit D</x:v>
       </x:c>
       <x:c r="E90" s="18" t="str">
-        <x:v>Administrasi</x:v>
+        <x:v>Pelatihan</x:v>
       </x:c>
       <x:c r="F90" s="18" t="str">
         <x:v>Belum Dimulai</x:v>
@@ -3710,7 +3720,7 @@
         <x:v>PIC-05</x:v>
       </x:c>
       <x:c r="J90" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K90" s="18" t="str">
         <x:v>Tidak ada catatan khusus</x:v>
@@ -3721,19 +3731,19 @@
         <x:v>AGD-0090</x:v>
       </x:c>
       <x:c r="B91" s="22" t="n">
-        <x:v>46224</x:v>
+        <x:v>46315</x:v>
       </x:c>
       <x:c r="C91" s="18" t="str">
-        <x:v>Pelatihan Internal</x:v>
+        <x:v>Kegiatan Administrasi</x:v>
       </x:c>
       <x:c r="D91" s="18" t="str">
         <x:v>Unit A</x:v>
       </x:c>
       <x:c r="E91" s="18" t="str">
-        <x:v>Rapat Internal</x:v>
+        <x:v>Administrasi</x:v>
       </x:c>
       <x:c r="F91" s="18" t="str">
-        <x:v>Selesai</x:v>
+        <x:v>Belum Dimulai</x:v>
       </x:c>
       <x:c r="G91" s="18" t="str">
         <x:v>Aula Kecamatan</x:v>
@@ -3745,7 +3755,7 @@
         <x:v>PIC-06</x:v>
       </x:c>
       <x:c r="J91" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K91" s="18" t="str">
         <x:v>Konfirmasi perlengkapan</x:v>
@@ -3756,7 +3766,7 @@
         <x:v>AGD-0091</x:v>
       </x:c>
       <x:c r="B92" s="22" t="n">
-        <x:v>46227</x:v>
+        <x:v>46316</x:v>
       </x:c>
       <x:c r="C92" s="18" t="str">
         <x:v>Rapat Koordinasi</x:v>
@@ -3765,10 +3775,10 @@
         <x:v>Unit B</x:v>
       </x:c>
       <x:c r="E92" s="18" t="str">
-        <x:v>Sosialisasi</x:v>
+        <x:v>Rapat Internal</x:v>
       </x:c>
       <x:c r="F92" s="18" t="str">
-        <x:v>Siap</x:v>
+        <x:v>Belum Dimulai</x:v>
       </x:c>
       <x:c r="G92" s="18" t="str">
         <x:v>Ruang Pelayanan</x:v>
@@ -3791,19 +3801,19 @@
         <x:v>AGD-0092</x:v>
       </x:c>
       <x:c r="B93" s="22" t="n">
-        <x:v>46230</x:v>
+        <x:v>46317</x:v>
       </x:c>
       <x:c r="C93" s="18" t="str">
-        <x:v>Evaluasi Bulanan</x:v>
+        <x:v>Sosialisasi Layanan</x:v>
       </x:c>
       <x:c r="D93" s="18" t="str">
         <x:v>Unit C</x:v>
       </x:c>
       <x:c r="E93" s="18" t="str">
-        <x:v>Evaluasi</x:v>
+        <x:v>Sosialisasi</x:v>
       </x:c>
       <x:c r="F93" s="18" t="str">
-        <x:v>Berjalan</x:v>
+        <x:v>Belum Dimulai</x:v>
       </x:c>
       <x:c r="G93" s="18" t="str">
         <x:v>Ruang Rapat 2</x:v>
@@ -3815,7 +3825,7 @@
         <x:v>PIC-08</x:v>
       </x:c>
       <x:c r="J93" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K93" s="18" t="str">
         <x:v>Data latihan</x:v>
@@ -3826,16 +3836,16 @@
         <x:v>AGD-0093</x:v>
       </x:c>
       <x:c r="B94" s="22" t="n">
-        <x:v>46233</x:v>
+        <x:v>46318</x:v>
       </x:c>
       <x:c r="C94" s="18" t="str">
-        <x:v>Kegiatan Administrasi</x:v>
+        <x:v>Evaluasi Bulanan</x:v>
       </x:c>
       <x:c r="D94" s="18" t="str">
         <x:v>Unit D</x:v>
       </x:c>
       <x:c r="E94" s="18" t="str">
-        <x:v>Pelatihan</x:v>
+        <x:v>Evaluasi</x:v>
       </x:c>
       <x:c r="F94" s="18" t="str">
         <x:v>Belum Dimulai</x:v>
@@ -3850,7 +3860,7 @@
         <x:v>PIC-09</x:v>
       </x:c>
       <x:c r="J94" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K94" s="18" t="str">
         <x:v>Tidak ada catatan khusus</x:v>
@@ -3861,19 +3871,19 @@
         <x:v>AGD-0094</x:v>
       </x:c>
       <x:c r="B95" s="22" t="n">
-        <x:v>46236</x:v>
+        <x:v>46319</x:v>
       </x:c>
       <x:c r="C95" s="18" t="str">
-        <x:v>Sosialisasi Layanan</x:v>
+        <x:v>Pelatihan Internal</x:v>
       </x:c>
       <x:c r="D95" s="18" t="str">
         <x:v>Unit A</x:v>
       </x:c>
       <x:c r="E95" s="18" t="str">
-        <x:v>Administrasi</x:v>
+        <x:v>Pelatihan</x:v>
       </x:c>
       <x:c r="F95" s="18" t="str">
-        <x:v>Selesai</x:v>
+        <x:v>Belum Dimulai</x:v>
       </x:c>
       <x:c r="G95" s="18" t="str">
         <x:v>Aula Kecamatan</x:v>
@@ -3896,19 +3906,19 @@
         <x:v>AGD-0095</x:v>
       </x:c>
       <x:c r="B96" s="22" t="n">
-        <x:v>46239</x:v>
+        <x:v>46320</x:v>
       </x:c>
       <x:c r="C96" s="18" t="str">
-        <x:v>Pelatihan Internal</x:v>
+        <x:v>Kegiatan Administrasi</x:v>
       </x:c>
       <x:c r="D96" s="18" t="str">
         <x:v>Unit B</x:v>
       </x:c>
       <x:c r="E96" s="18" t="str">
-        <x:v>Rapat Internal</x:v>
+        <x:v>Administrasi</x:v>
       </x:c>
       <x:c r="F96" s="18" t="str">
-        <x:v>Siap</x:v>
+        <x:v>Belum Dimulai</x:v>
       </x:c>
       <x:c r="G96" s="18" t="str">
         <x:v>Ruang Pelayanan</x:v>
@@ -3920,7 +3930,7 @@
         <x:v>PIC-11</x:v>
       </x:c>
       <x:c r="J96" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K96" s="18" t="str">
         <x:v>Menunggu jadwal final</x:v>
@@ -3931,7 +3941,7 @@
         <x:v>AGD-0096</x:v>
       </x:c>
       <x:c r="B97" s="22" t="n">
-        <x:v>46242</x:v>
+        <x:v>46321</x:v>
       </x:c>
       <x:c r="C97" s="18" t="str">
         <x:v>Rapat Koordinasi</x:v>
@@ -3940,10 +3950,10 @@
         <x:v>Unit C</x:v>
       </x:c>
       <x:c r="E97" s="18" t="str">
-        <x:v>Sosialisasi</x:v>
+        <x:v>Rapat Internal</x:v>
       </x:c>
       <x:c r="F97" s="18" t="str">
-        <x:v>Berjalan</x:v>
+        <x:v>Belum Dimulai</x:v>
       </x:c>
       <x:c r="G97" s="18" t="str">
         <x:v>Ruang Rapat 2</x:v>
@@ -3955,7 +3965,7 @@
         <x:v>PIC-12</x:v>
       </x:c>
       <x:c r="J97" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K97" s="18" t="str">
         <x:v>Data latihan</x:v>
@@ -3966,16 +3976,16 @@
         <x:v>AGD-0097</x:v>
       </x:c>
       <x:c r="B98" s="22" t="n">
-        <x:v>46245</x:v>
+        <x:v>46322</x:v>
       </x:c>
       <x:c r="C98" s="18" t="str">
-        <x:v>Evaluasi Bulanan</x:v>
+        <x:v>Sosialisasi Layanan</x:v>
       </x:c>
       <x:c r="D98" s="18" t="str">
         <x:v>Unit D</x:v>
       </x:c>
       <x:c r="E98" s="18" t="str">
-        <x:v>Evaluasi</x:v>
+        <x:v>Sosialisasi</x:v>
       </x:c>
       <x:c r="F98" s="18" t="str">
         <x:v>Belum Dimulai</x:v>
@@ -4001,19 +4011,19 @@
         <x:v>AGD-0098</x:v>
       </x:c>
       <x:c r="B99" s="22" t="n">
-        <x:v>46248</x:v>
+        <x:v>46323</x:v>
       </x:c>
       <x:c r="C99" s="18" t="str">
-        <x:v>Kegiatan Administrasi</x:v>
+        <x:v>Evaluasi Bulanan</x:v>
       </x:c>
       <x:c r="D99" s="18" t="str">
         <x:v>Unit A</x:v>
       </x:c>
       <x:c r="E99" s="18" t="str">
-        <x:v>Pelatihan</x:v>
+        <x:v>Evaluasi</x:v>
       </x:c>
       <x:c r="F99" s="18" t="str">
-        <x:v>Selesai</x:v>
+        <x:v>Belum Dimulai</x:v>
       </x:c>
       <x:c r="G99" s="18" t="str">
         <x:v>Aula Kecamatan</x:v>
@@ -4025,7 +4035,7 @@
         <x:v>PIC-02</x:v>
       </x:c>
       <x:c r="J99" s="18" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Sedang</x:v>
       </x:c>
       <x:c r="K99" s="18" t="str">
         <x:v>Konfirmasi perlengkapan</x:v>
@@ -4036,19 +4046,19 @@
         <x:v>AGD-0099</x:v>
       </x:c>
       <x:c r="B100" s="22" t="n">
-        <x:v>46251</x:v>
+        <x:v>46324</x:v>
       </x:c>
       <x:c r="C100" s="18" t="str">
-        <x:v>Sosialisasi Layanan</x:v>
+        <x:v>Pelatihan Internal</x:v>
       </x:c>
       <x:c r="D100" s="18" t="str">
         <x:v>Unit B</x:v>
       </x:c>
       <x:c r="E100" s="18" t="str">
-        <x:v>Administrasi</x:v>
+        <x:v>Pelatihan</x:v>
       </x:c>
       <x:c r="F100" s="18" t="str">
-        <x:v>Siap</x:v>
+        <x:v>Belum Dimulai</x:v>
       </x:c>
       <x:c r="G100" s="18" t="str">
         <x:v>Ruang Pelayanan</x:v>
@@ -4060,7 +4070,7 @@
         <x:v>PIC-03</x:v>
       </x:c>
       <x:c r="J100" s="18" t="str">
-        <x:v>Sedang</x:v>
+        <x:v>Normal</x:v>
       </x:c>
       <x:c r="K100" s="18" t="str">
         <x:v>Menunggu jadwal final</x:v>
@@ -4071,19 +4081,19 @@
         <x:v>AGD-0100</x:v>
       </x:c>
       <x:c r="B101" s="23" t="n">
-        <x:v>46254</x:v>
+        <x:v>46325</x:v>
       </x:c>
       <x:c r="C101" s="20" t="str">
-        <x:v>Pelatihan Internal</x:v>
+        <x:v>Kegiatan Administrasi</x:v>
       </x:c>
       <x:c r="D101" s="20" t="str">
         <x:v>Unit C</x:v>
       </x:c>
       <x:c r="E101" s="20" t="str">
-        <x:v>Rapat Internal</x:v>
+        <x:v>Administrasi</x:v>
       </x:c>
       <x:c r="F101" s="20" t="str">
-        <x:v>Berjalan</x:v>
+        <x:v>Belum Dimulai</x:v>
       </x:c>
       <x:c r="G101" s="20" t="str">
         <x:v>Ruang Rapat 2</x:v>
@@ -4104,7 +4114,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R635b41874e044227"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f36c52c424344af"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4161,14 +4171,14 @@
       </x:c>
     </x:row>
     <x:row r="7" ht="38" customHeight="1">
-      <x:c r="A7" s="44" t="str">
-        <x:v>Catatan</x:v>
+      <x:c r="A7" s="43" t="str">
+        <x:v>Tanggal</x:v>
       </x:c>
       <x:c r="B7" s="43" t="str">
-        <x:v>2026-03-12</x:v>
+        <x:v>2026-10-12</x:v>
       </x:c>
       <x:c r="C7" s="43" t="str">
-        <x:v>Tanggal pelaksanaan atau target kegiatan.</x:v>
+        <x:v>Tanggal pelaksanaan/target kegiatan. Status latihan dibuat konsisten dengan tanggal acuan 2026-10-04.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="38" customHeight="1">
@@ -4269,11 +4279,19 @@
       <x:c r="C16" s="43" t="str">
         <x:v>Catatan umum untuk persiapan kegiatan.</x:v>
       </x:c>
+    </x:row>
+    <x:row r="17" ht="34" customHeight="1">
+      <x:c r="A17" s="47" t="str">
+        <x:v>Catatan: gunakan data sintetis selama latihan dan jangan memasukkan data pribadi ke ChatGPT.</x:v>
+      </x:c>
+      <x:c r="B17" s="47"/>
+      <x:c r="C17" s="47"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>
     <x:mergeCell ref="A3:F3"/>
+    <x:mergeCell ref="A17:C17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>